<commit_message>
removed "Pset_" name, due to BuildingSmart reserve it for standard Psets. Ours is now "BEGEES_"
</commit_message>
<xml_diff>
--- a/Detaljplan2IFC/schema.xlsx
+++ b/Detaljplan2IFC/schema.xlsx
@@ -775,10 +775,11 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Pset_DetaljplanBestammelse</t>
-        </is>
-      </c>
-    </row>
+          <t>BEGEES_DetaljplanBestammelse</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>

</xml_diff>